<commit_message>
chore(CWL): update TinyMita example
</commit_message>
<xml_diff>
--- a/CwlExamples/TinyMita/LangMod/EN/Dialog/dialog.xlsx
+++ b/CwlExamples/TinyMita/LangMod/EN/Dialog/dialog.xlsx
@@ -5,18 +5,21 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Program Files (x86)\Steam\steamapps\common\Elin\Package\Mod_TinyMita\LangMod\EN\Dialog\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SteamLibrary\steamapps\common\Elin\Package\Mod_TinyMita\LangMod\EN\Dialog\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6106F20B-D9EF-48C5-8371-A78D9806F47F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{287D4ED9-86A9-40F7-903C-8C1ECE2034A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="51480" yWindow="5205" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20925" yWindow="2760" windowWidth="26940" windowHeight="17625" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="unique" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="CalcA1"/>
     </ext>
@@ -25,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
   <si>
     <t>id</t>
   </si>
@@ -55,6 +58,24 @@
 いっしょにあそぼうよ…
 ねえ、プレイヤー…</t>
     <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>你为什么要离开？
+留下来…
+我们一起玩吧！
+玩家…</t>
+  </si>
+  <si>
+    <t>text_CN</t>
+  </si>
+  <si>
+    <t>text_ZHTW</t>
+  </si>
+  <si>
+    <t>你為什麼要離開？
+留下來…
+我們一起玩吧！
+玩家…</t>
   </si>
 </sst>
 </file>
@@ -120,7 +141,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
@@ -130,9 +151,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -325,16 +349,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D33"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="16.5"/>
   <cols>
     <col min="1" max="1" width="14.5703125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="111" style="1" customWidth="1"/>
-    <col min="4" max="4" width="87.140625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="19.28515625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="39" style="1" customWidth="1"/>
+    <col min="4" max="4" width="22.5703125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="18.85546875" customWidth="1"/>
+    <col min="6" max="6" width="23.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -347,68 +373,83 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4">
+      <c r="E1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
       <c r="C2" s="3"/>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:6">
       <c r="C3" s="3"/>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:6">
       <c r="C4" s="3"/>
     </row>
-    <row r="5" spans="1:4" ht="66">
+    <row r="5" spans="1:6" ht="82.5">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
+      <c r="B5" s="3" t="s">
+        <v>5</v>
+      </c>
       <c r="C5" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="6" spans="1:4">
+      <c r="E5" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:6">
       <c r="C7" s="3"/>
       <c r="D7" s="3"/>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:6">
       <c r="C8" s="3"/>
       <c r="D8" s="3"/>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:6">
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:6">
       <c r="C10" s="3"/>
       <c r="D10" s="3"/>
     </row>
-    <row r="11" spans="1:4">
+    <row r="11" spans="1:6">
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
     </row>
-    <row r="12" spans="1:4">
+    <row r="12" spans="1:6">
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
     </row>
-    <row r="13" spans="1:4">
+    <row r="13" spans="1:6">
       <c r="C13" s="3"/>
     </row>
-    <row r="14" spans="1:4">
+    <row r="14" spans="1:6">
       <c r="C14" s="3"/>
       <c r="D14" s="3"/>
     </row>
-    <row r="15" spans="1:4">
+    <row r="15" spans="1:6">
       <c r="C15" s="3"/>
       <c r="D15" s="3"/>
     </row>
-    <row r="16" spans="1:4">
+    <row r="16" spans="1:6">
       <c r="C16" s="3"/>
       <c r="D16" s="3"/>
     </row>

</xml_diff>